<commit_message>
gradebook updated for ddm
</commit_message>
<xml_diff>
--- a/materials/GradeBook.xlsx
+++ b/materials/GradeBook.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\STUDY\SWIN\Lab\JDA\V&amp;V\validation4llmagents\materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8EBA430-EA7C-4BAE-91FC-67E2E453DE3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0298A85D-E94D-45AF-A7A9-E8E0CA66C8EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{42BDA58E-0774-40FA-86BF-817CBA65D2BA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="3" xr2:uid="{42BDA58E-0774-40FA-86BF-817CBA65D2BA}"/>
   </bookViews>
   <sheets>
     <sheet name="Docs" sheetId="3" r:id="rId1"/>
     <sheet name="Model 1" sheetId="1" r:id="rId2"/>
     <sheet name="Model 2" sheetId="2" r:id="rId3"/>
+    <sheet name="Requirements" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="36">
   <si>
     <t>ReqID_g</t>
   </si>
@@ -103,12 +104,6 @@
     <t>Number of gold elements (actions, branches, transitions) semantically matched by the agent / Total number of gold elements</t>
   </si>
   <si>
-    <t>VMX Requirement Coverage</t>
-  </si>
-  <si>
-    <t>Number of requirements linked to at least one source input, class element, or activity element in the VMX / Total number of requirements</t>
-  </si>
-  <si>
     <t>Requirement Precision</t>
   </si>
   <si>
@@ -127,18 +122,6 @@
     <t>Number of generated elements (actions, branches, transitions) judged semantically correct / Total number of generated elements</t>
   </si>
   <si>
-    <t>Syntax Validity</t>
-  </si>
-  <si>
-    <t>Number of syntactically valid elements / Total number of elements</t>
-  </si>
-  <si>
-    <t>VMX Referential Integrity</t>
-  </si>
-  <si>
-    <t>Number of VMX references that point to existing items / Total number of VMX references</t>
-  </si>
-  <si>
     <t>Model 1: TP/(TP + FN)</t>
   </si>
   <si>
@@ -151,9 +134,6 @@
     <t>Model 1 + Model 2 TP/(TP + FN)</t>
   </si>
   <si>
-    <t>?</t>
-  </si>
-  <si>
     <t>Sem</t>
   </si>
   <si>
@@ -167,9 +147,6 @@
   </si>
   <si>
     <t>Model 2 Sem/Total generated elements</t>
-  </si>
-  <si>
-    <t>Model 1 + Model 2 Syn/ Total generated elements</t>
   </si>
 </sst>
 </file>
@@ -231,7 +208,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -278,24 +255,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -308,7 +272,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -322,9 +286,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -661,7 +622,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB5346A6-1B10-474A-AFB1-2FE4F9168116}">
-  <dimension ref="A2:D13"/>
+  <dimension ref="A2:D10"/>
   <sheetFormatPr defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
@@ -678,7 +639,7 @@
         <v>12</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>13</v>
@@ -695,7 +656,7 @@
         <v>16</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="60">
@@ -707,7 +668,7 @@
         <v>18</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="60">
@@ -719,11 +680,13 @@
         <v>20</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="60">
-      <c r="A6" s="12"/>
+      <c r="A6" s="10" t="s">
+        <v>10</v>
+      </c>
       <c r="B6" s="8" t="s">
         <v>21</v>
       </c>
@@ -731,13 +694,11 @@
         <v>22</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="60">
-      <c r="A7" s="10" t="s">
-        <v>10</v>
-      </c>
+      <c r="A7" s="11"/>
       <c r="B7" s="8" t="s">
         <v>23</v>
       </c>
@@ -745,7 +706,7 @@
         <v>24</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="60">
@@ -757,52 +718,16 @@
         <v>26</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="60">
-      <c r="A9" s="11"/>
-      <c r="B9" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="30">
-      <c r="A10" s="11"/>
-      <c r="B10" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="45">
-      <c r="A11" s="12"/>
-      <c r="B11" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="B13" s="6"/>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="B10" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="A7:A11"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="A6:A8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -843,10 +768,10 @@
         <v>7</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="K1" s="1"/>
     </row>
@@ -892,10 +817,10 @@
         <v>7</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:10">
@@ -951,6 +876,42 @@
     </row>
     <row r="19" spans="1:1" ht="15.6">
       <c r="A19" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2A1650-03E9-4C68-A4D3-706C9A8E7E33}">
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr defaultRowHeight="15.6"/>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>